<commit_message>
Add SOH report for 2026-10-19
</commit_message>
<xml_diff>
--- a/reports/SOH_18_10_2026.xlsx
+++ b/reports/SOH_18_10_2026.xlsx
@@ -993,7 +993,7 @@
         </is>
       </c>
       <c r="D20" s="2" t="n">
-        <v>568</v>
+        <v>567</v>
       </c>
       <c r="E20" s="3" t="n">
         <v>0</v>
@@ -1301,7 +1301,7 @@
         </is>
       </c>
       <c r="D31" s="2" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E31" s="3" t="n">
         <v>40000</v>
@@ -1553,7 +1553,7 @@
         </is>
       </c>
       <c r="D40" s="2" t="n">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="E40" s="3" t="n">
         <v>21000</v>
@@ -1665,7 +1665,7 @@
         </is>
       </c>
       <c r="D44" s="2" t="n">
-        <v>559</v>
+        <v>556</v>
       </c>
       <c r="E44" s="3" t="n">
         <v>4500</v>
@@ -2029,7 +2029,7 @@
         </is>
       </c>
       <c r="D57" s="2" t="n">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="E57" s="3" t="n">
         <v>51000</v>
@@ -2169,7 +2169,7 @@
         </is>
       </c>
       <c r="D62" s="2" t="n">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="E62" s="3" t="n">
         <v>51000</v>
@@ -2533,7 +2533,7 @@
         </is>
       </c>
       <c r="D75" s="2" t="n">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E75" s="3" t="n">
         <v>4000</v>
@@ -2561,7 +2561,7 @@
         </is>
       </c>
       <c r="D76" s="2" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="E76" s="3" t="n">
         <v>4000</v>
@@ -2813,7 +2813,7 @@
         </is>
       </c>
       <c r="D85" s="2" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="E85" s="3" t="n">
         <v>20000</v>
@@ -3009,7 +3009,7 @@
         </is>
       </c>
       <c r="D92" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E92" s="3" t="n">
         <v>8000</v>
@@ -3093,7 +3093,7 @@
         </is>
       </c>
       <c r="D95" s="2" t="n">
-        <v>455</v>
+        <v>454</v>
       </c>
       <c r="E95" s="3" t="n">
         <v>7612</v>
@@ -3457,7 +3457,7 @@
         </is>
       </c>
       <c r="D108" s="2" t="n">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="E108" s="3" t="n">
         <v>1</v>
@@ -3485,7 +3485,7 @@
         </is>
       </c>
       <c r="D109" s="2" t="n">
-        <v>2613</v>
+        <v>2596</v>
       </c>
       <c r="E109" s="3" t="n">
         <v>3876</v>
@@ -3793,7 +3793,7 @@
         </is>
       </c>
       <c r="D120" s="2" t="n">
-        <v>2043</v>
+        <v>2041</v>
       </c>
       <c r="E120" s="3" t="n">
         <v>3800</v>
@@ -4713,7 +4713,7 @@
         </is>
       </c>
       <c r="D153" s="2" t="n">
-        <v>440</v>
+        <v>438</v>
       </c>
       <c r="E153" s="3" t="n">
         <v>1</v>
@@ -4741,7 +4741,7 @@
         </is>
       </c>
       <c r="D154" s="2" t="n">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="E154" s="3" t="n">
         <v>1</v>
@@ -4853,7 +4853,7 @@
         </is>
       </c>
       <c r="D158" s="2" t="n">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="E158" s="3" t="n">
         <v>1</v>
@@ -5393,7 +5393,7 @@
         </is>
       </c>
       <c r="D178" s="2" t="n">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="E178" s="3" t="n">
         <v>1</v>
@@ -6713,7 +6713,7 @@
         </is>
       </c>
       <c r="D227" s="2" t="n">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="E227" s="3" t="n">
         <v>1</v>
@@ -9850,7 +9850,7 @@
         </is>
       </c>
       <c r="D340" s="2" t="n">
-        <v>472</v>
+        <v>88</v>
       </c>
       <c r="E340" s="3" t="n">
         <v>2500</v>
@@ -10102,7 +10102,7 @@
         </is>
       </c>
       <c r="D349" s="2" t="n">
-        <v>194</v>
+        <v>122</v>
       </c>
       <c r="E349" s="3" t="n">
         <v>6376</v>
@@ -10942,7 +10942,7 @@
         </is>
       </c>
       <c r="D379" s="2" t="n">
-        <v>73</v>
+        <v>63</v>
       </c>
       <c r="E379" s="3" t="n">
         <v>39772</v>
@@ -15534,7 +15534,7 @@
         </is>
       </c>
       <c r="D543" s="2" t="n">
-        <v>324</v>
+        <v>278</v>
       </c>
       <c r="E543" s="3" t="n">
         <v>12816</v>
@@ -16290,7 +16290,7 @@
         </is>
       </c>
       <c r="D570" s="2" t="n">
-        <v>238</v>
+        <v>214</v>
       </c>
       <c r="E570" s="3" t="n">
         <v>10491</v>
@@ -16962,7 +16962,7 @@
         </is>
       </c>
       <c r="D594" s="2" t="n">
-        <v>1139</v>
+        <v>1133</v>
       </c>
       <c r="E594" s="3" t="n">
         <v>19364</v>
@@ -17943,7 +17943,7 @@
         </is>
       </c>
       <c r="D629" s="2" t="n">
-        <v>3755</v>
+        <v>3683</v>
       </c>
       <c r="E629" s="3" t="n">
         <v>10251</v>
@@ -17971,7 +17971,7 @@
         </is>
       </c>
       <c r="D630" s="2" t="n">
-        <v>149</v>
+        <v>101</v>
       </c>
       <c r="E630" s="3" t="n">
         <v>12094</v>
@@ -18839,7 +18839,7 @@
         </is>
       </c>
       <c r="D661" s="2" t="n">
-        <v>899</v>
+        <v>803</v>
       </c>
       <c r="E661" s="3" t="n">
         <v>15053</v>
@@ -18951,7 +18951,7 @@
         </is>
       </c>
       <c r="D665" s="2" t="n">
-        <v>169</v>
+        <v>73</v>
       </c>
       <c r="E665" s="3" t="n">
         <v>13716</v>
@@ -19595,7 +19595,7 @@
         </is>
       </c>
       <c r="D688" s="2" t="n">
-        <v>215</v>
+        <v>191</v>
       </c>
       <c r="E688" s="3" t="n">
         <v>8577</v>
@@ -21583,7 +21583,7 @@
         </is>
       </c>
       <c r="D759" s="2" t="n">
-        <v>671</v>
+        <v>335</v>
       </c>
       <c r="E759" s="3" t="n">
         <v>17475</v>
@@ -22087,7 +22087,7 @@
         </is>
       </c>
       <c r="D777" s="2" t="n">
-        <v>233</v>
+        <v>221</v>
       </c>
       <c r="E777" s="3" t="n">
         <v>5157</v>
@@ -24103,7 +24103,7 @@
         </is>
       </c>
       <c r="D849" s="2" t="n">
-        <v>204</v>
+        <v>84</v>
       </c>
       <c r="E849" s="3" t="n">
         <v>6669</v>
@@ -25252,7 +25252,7 @@
         </is>
       </c>
       <c r="D890" s="2" t="n">
-        <v>68</v>
+        <v>20</v>
       </c>
       <c r="E890" s="3" t="n">
         <v>5514</v>
@@ -25868,7 +25868,7 @@
         </is>
       </c>
       <c r="D912" s="2" t="n">
-        <v>102</v>
+        <v>66</v>
       </c>
       <c r="E912" s="3" t="n">
         <v>9284</v>
@@ -25953,7 +25953,7 @@
         </is>
       </c>
       <c r="D915" s="2" t="n">
-        <v>1348</v>
+        <v>1300</v>
       </c>
       <c r="E915" s="3" t="n">
         <v>8181</v>
@@ -26121,7 +26121,7 @@
         </is>
       </c>
       <c r="D921" s="2" t="n">
-        <v>181</v>
+        <v>157</v>
       </c>
       <c r="E921" s="3" t="n">
         <v>11577</v>
@@ -27664,7 +27664,7 @@
         </is>
       </c>
       <c r="D976" s="2" t="n">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="E976" s="3" t="n">
         <v>8700</v>
@@ -30156,7 +30156,7 @@
         </is>
       </c>
       <c r="D1065" s="2" t="n">
-        <v>280</v>
+        <v>232</v>
       </c>
       <c r="E1065" s="3" t="n">
         <v>13520</v>
@@ -30548,7 +30548,7 @@
         </is>
       </c>
       <c r="D1079" s="2" t="n">
-        <v>135</v>
+        <v>27</v>
       </c>
       <c r="E1079" s="3" t="n">
         <v>8060</v>
@@ -31977,7 +31977,7 @@
         </is>
       </c>
       <c r="D1130" s="2" t="n">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="E1130" s="3" t="n">
         <v>10691</v>
@@ -32145,7 +32145,7 @@
         </is>
       </c>
       <c r="D1136" s="2" t="n">
-        <v>233</v>
+        <v>209</v>
       </c>
       <c r="E1136" s="3" t="n">
         <v>14451</v>
@@ -33237,7 +33237,7 @@
         </is>
       </c>
       <c r="D1175" s="2" t="n">
-        <v>645</v>
+        <v>549</v>
       </c>
       <c r="E1175" s="3" t="n">
         <v>11372</v>
@@ -34385,7 +34385,7 @@
         </is>
       </c>
       <c r="D1216" s="2" t="n">
-        <v>70</v>
+        <v>22</v>
       </c>
       <c r="E1216" s="3" t="n">
         <v>14752</v>
@@ -34525,7 +34525,7 @@
         </is>
       </c>
       <c r="D1221" s="2" t="n">
-        <v>409</v>
+        <v>313</v>
       </c>
       <c r="E1221" s="3" t="n">
         <v>8325</v>
@@ -35785,7 +35785,7 @@
         </is>
       </c>
       <c r="D1266" s="2" t="n">
-        <v>100</v>
+        <v>94</v>
       </c>
       <c r="E1266" s="3" t="n">
         <v>16160</v>
@@ -35953,7 +35953,7 @@
         </is>
       </c>
       <c r="D1272" s="2" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="E1272" s="3" t="n">
         <v>5601</v>
@@ -36121,7 +36121,7 @@
         </is>
       </c>
       <c r="D1278" s="2" t="n">
-        <v>116</v>
+        <v>91</v>
       </c>
       <c r="E1278" s="3" t="n">
         <v>6594</v>
@@ -36233,7 +36233,7 @@
         </is>
       </c>
       <c r="D1282" s="2" t="n">
-        <v>108</v>
+        <v>84</v>
       </c>
       <c r="E1282" s="3" t="n">
         <v>8855</v>
@@ -36429,7 +36429,7 @@
         </is>
       </c>
       <c r="D1289" s="2" t="n">
-        <v>11</v>
+        <v>-1</v>
       </c>
       <c r="E1289" s="3" t="n">
         <v>27857</v>
@@ -36513,7 +36513,7 @@
         </is>
       </c>
       <c r="D1292" s="2" t="n">
-        <v>73</v>
+        <v>79</v>
       </c>
       <c r="E1292" s="3" t="n">
         <v>15804</v>
@@ -36821,7 +36821,7 @@
         </is>
       </c>
       <c r="D1303" s="2" t="n">
-        <v>324</v>
+        <v>276</v>
       </c>
       <c r="E1303" s="3" t="n">
         <v>6603</v>
@@ -37493,7 +37493,7 @@
         </is>
       </c>
       <c r="D1327" s="2" t="n">
-        <v>1025</v>
+        <v>881</v>
       </c>
       <c r="E1327" s="3" t="n">
         <v>5882</v>
@@ -37605,7 +37605,7 @@
         </is>
       </c>
       <c r="D1331" s="2" t="n">
-        <v>112</v>
+        <v>40</v>
       </c>
       <c r="E1331" s="3" t="n">
         <v>36976</v>
@@ -37633,7 +37633,7 @@
         </is>
       </c>
       <c r="D1332" s="2" t="n">
-        <v>75</v>
+        <v>0</v>
       </c>
       <c r="E1332" s="3" t="n">
         <v>23875</v>
@@ -37745,7 +37745,7 @@
         </is>
       </c>
       <c r="D1336" s="2" t="n">
-        <v>270</v>
+        <v>198</v>
       </c>
       <c r="E1336" s="3" t="n">
         <v>13720</v>
@@ -38221,7 +38221,7 @@
         </is>
       </c>
       <c r="D1353" s="2" t="n">
-        <v>440</v>
+        <v>368</v>
       </c>
       <c r="E1353" s="3" t="n">
         <v>25495</v>
@@ -38305,7 +38305,7 @@
         </is>
       </c>
       <c r="D1356" s="2" t="n">
-        <v>436</v>
+        <v>388</v>
       </c>
       <c r="E1356" s="3" t="n">
         <v>8246</v>
@@ -39565,7 +39565,7 @@
         </is>
       </c>
       <c r="D1401" s="2" t="n">
-        <v>231</v>
+        <v>225</v>
       </c>
       <c r="E1401" s="3" t="n">
         <v>5674</v>
@@ -39789,7 +39789,7 @@
         </is>
       </c>
       <c r="D1409" s="2" t="n">
-        <v>767</v>
+        <v>743</v>
       </c>
       <c r="E1409" s="3" t="n">
         <v>7174</v>
@@ -40433,7 +40433,7 @@
         </is>
       </c>
       <c r="D1432" s="2" t="n">
-        <v>1225</v>
+        <v>1201</v>
       </c>
       <c r="E1432" s="3" t="n">
         <v>14093</v>
@@ -41021,7 +41021,7 @@
         </is>
       </c>
       <c r="D1453" s="2" t="n">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="E1453" s="3" t="n">
         <v>30208</v>
@@ -43429,7 +43429,7 @@
         </is>
       </c>
       <c r="D1539" s="2" t="n">
-        <v>487</v>
+        <v>207</v>
       </c>
       <c r="E1539" s="3" t="n">
         <v>12419</v>
@@ -46090,7 +46090,7 @@
         </is>
       </c>
       <c r="D1634" s="2" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="E1634" s="3" t="n">
         <v>8238</v>

</xml_diff>